<commit_message>
fix: harden Hanoi formula inputs
</commit_message>
<xml_diff>
--- a/Hanoi/Hanoi-1.0.xlsx
+++ b/Hanoi/Hanoi-1.0.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Hanoi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE1E9FAE-DED2-5045-8564-EC09F255659E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA7E69D7-A897-114E-A520-10216280EA7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="17300" xr2:uid="{82D447F9-66A8-4F40-88AB-946121063596}"/>
+    <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15900" xr2:uid="{82D447F9-66A8-4F40-88AB-946121063596}"/>
   </bookViews>
   <sheets>
     <sheet name="Stage" sheetId="2" r:id="rId1"/>
@@ -24,10 +24,10 @@
     <definedName name="HanoiDisks">Stage!$B$5</definedName>
     <definedName name="HanoiMaxStep">Engine!$B$6</definedName>
     <definedName name="HanoiStep">Stage!$B$6</definedName>
-    <definedName name="HN_CLAMP_DISKS">_xlfn.LAMBDA(_xlpm.n,MAX(1,MIN(6,_xlpm.n)))</definedName>
+    <definedName name="HN_CLAMP_DISKS">_xlfn.LAMBDA(_xlpm.n,_xlfn.LET(_xlpm.v,IFERROR(--_xlpm.n,3),MAX(3,MIN(6,ROUND(_xlpm.v,0)))))</definedName>
     <definedName name="HN_CURRENT_MOVE">_xlfn.LAMBDA(_xlpm.step,IF(_xlpm.step=0,"Start Pose","Step "&amp;_xlpm.step&amp;": "&amp;HN_MOVE_LABEL(_xlpm.step," ")))</definedName>
     <definedName name="HN_DISK_POS">_xlfn.LAMBDA(_xlpm.step,_xlpm.n,_xlpm.d,_xlpm.maxStep,IF(AND(_xlpm.step&lt;=_xlpm.maxStep,_xlpm.d&lt;=_xlpm.n),1+MOD(IF(MOD(_xlpm.n-_xlpm.d,2)=0,-1,1)*QUOTIENT(_xlpm.step+2^(_xlpm.d-1),2^_xlpm.d),3),""))</definedName>
-    <definedName name="HN_EFFECTIVE_STEP">_xlfn.LAMBDA(_xlpm.inputStep,_xlpm.maxStep,MAX(0,MIN(_xlpm.inputStep,_xlpm.maxStep)))</definedName>
+    <definedName name="HN_EFFECTIVE_STEP">_xlfn.LAMBDA(_xlpm.inputStep,_xlpm.maxStep,_xlfn.LET(_xlpm.v,IFERROR(--_xlpm.inputStep,0),MAX(0,MIN(_xlpm.maxStep,ROUND(_xlpm.v,0)))))</definedName>
     <definedName name="HN_KEYFRAME_STEP">_xlfn.LAMBDA(_xlpm.cur,_xlpm.maxs,_xlpm.rowOffset,_xlfn.LET(_xlpm.win,7,_xlpm.start,MAX(0,MIN(_xlpm.maxs-_xlpm.win,_xlpm.cur-3)),_xlpm.start+_xlpm.rowOffset))</definedName>
     <definedName name="HN_LOCAL">_xlfn.LAMBDA(_xlpm.g,_xlpm.peg,IF(_xlpm.peg=1,_xlpm.g-1,IF(_xlpm.peg=2,_xlpm.g-13,IF(_xlpm.peg=3,_xlpm.g-25,0))))</definedName>
     <definedName name="HN_MAX_STEP">_xlfn.LAMBDA(_xlpm.n,2^_xlpm.n-1)</definedName>
@@ -41,7 +41,7 @@
     <definedName name="HN_PEG_LABEL">_xlfn.LAMBDA(_xlpm.p,IF(_xlpm.p="","",CHOOSE(_xlpm.p,"A","B","C")))</definedName>
     <definedName name="HN_POS_ROW">_xlfn.LAMBDA(_xlpm.step,_xlfn.XLOOKUP(_xlpm.step,Engine!$A$11:$A$74,Engine!$F$11:$K$74,""))</definedName>
     <definedName name="HN_POSITIONS">_xlfn.LAMBDA(_xlpm.n,_xlpm.curRange,_xlfn.TEXTJOIN("  ",TRUE,_xlfn.MAP(_xlfn.SEQUENCE(1,_xlpm.n),_xlfn.LAMBDA(_xlpm.d,"D"&amp;_xlpm.d&amp;":"&amp;CHOOSE(INDEX(_xlpm.curRange,1,_xlpm.d),"A","B","C")))))</definedName>
-    <definedName name="HN_PROGRESS_BAR">_xlfn.LAMBDA(_xlpm.step,_xlpm.maxs,_xlpm.bins,_xlfn.LET(_xlpm.fill,IF(_xlpm.maxs=0,0,ROUND(_xlpm.step/_xlpm.maxs*_xlpm.bins,0)),REPT("■",_xlpm.fill)&amp;REPT("□",_xlpm.bins-_xlpm.fill)&amp;"  "&amp;_xlpm.fill&amp;"/"&amp;_xlpm.bins))</definedName>
+    <definedName name="HN_PROGRESS_BAR">_xlfn.LAMBDA(_xlpm.step,_xlpm.maxs,_xlpm.bins,_xlfn.LET(_xlpm.fill,IF(_xlpm.maxs=0,0,ROUND(_xlpm.step/_xlpm.maxs*_xlpm.bins,0)),_xlpm.pct,IF(_xlpm.maxs=0,0,_xlpm.step/_xlpm.maxs),REPT("■",_xlpm.fill)&amp;REPT("□",_xlpm.bins-_xlpm.fill)&amp;"  "&amp;TEXT(_xlpm.pct,"0%")))</definedName>
     <definedName name="HN_STAGE_CELL">_xlfn.LAMBDA(_xlpm.g,_xlpm.r,_xlpm.n,_xlpm.curRange,_xlfn.LET(_xlpm.m,6,_xlpm.all,_xlfn.SEQUENCE(1,_xlpm.n),_xlpm.cur,INDEX(_xlpm.curRange,1,_xlpm.all),_xlpm.peg,HN_PEG(_xlpm.g),_xlpm.local,HN_LOCAL(_xlpm.g,_xlpm.peg),_xlpm.center,6,_xlpm.k,IF(_xlpm.peg=0,0,SUM(--(_xlpm.cur=_xlpm.peg))),_xlpm.idx,_xlpm.r-(_xlpm.m-_xlpm.k),_xlpm.staticDisks,IF(_xlpm.peg=0,"",_xlfn._xlws.FILTER(_xlpm.all,_xlpm.cur=_xlpm.peg,"")),_xlpm.d,IF(OR(_xlpm.peg=0,_xlpm.idx&lt;1),"",IFERROR(INDEX(_xlpm.staticDisks,1,_xlpm.idx),"")),_xlpm.mark,IF(_xlpm.d="","","█"),IF(_xlpm.r&lt;=_xlpm.m,IF(_xlpm.peg=0," ",IF(_xlpm.d="",IF(_xlpm.local=_xlpm.center,"│"," "),IF(ABS(_xlpm.local-_xlpm.center)&lt;=_xlpm.d-1,_xlpm.mark," "))),IF(_xlpm.r=_xlpm.m+1,IF(_xlpm.peg=0," ","─"),IF(_xlpm.r=_xlpm.m+2,IF(AND(_xlpm.peg&lt;&gt;0,_xlpm.local=_xlpm.center),CHOOSE(_xlpm.peg,"A","B","C")," "),"")))))</definedName>
     <definedName name="HN_STAGE_TITLE">_xlfn.LAMBDA(_xlpm.step,_xlpm.n,IF(_xlpm.step=0,"Motion Stage · Step 0 / "&amp;HN_MAX_STEP(_xlpm.n)&amp;" · Start Pose","Motion Stage · Step "&amp;_xlpm.step&amp;" / "&amp;HN_MAX_STEP(_xlpm.n)&amp;" · "&amp;HN_MOVE_LABEL(_xlpm.step," ")))</definedName>
     <definedName name="HN_STEP_LIST">_xlfn.LAMBDA(_xlpm.maxStep,_xlfn.SEQUENCE(_xlpm.maxStep+1,1,0,1))</definedName>
@@ -642,11 +642,68 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Derived source peg for the moving disk at each step. Feeds Sheet2 Status and Keyframes.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E18" authorId="0" shapeId="0" xr:uid="{242B9B47-8033-9044-92CB-22DFD00ACA15}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Yuan Jiang:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Derived destination peg for the moving disk at each step. Feeds Sheet2 Status and Keyframes.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D19" authorId="0" shapeId="0" xr:uid="{600C42A8-8DDE-F946-A285-12B72DF5D886}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Yuan Jiang:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 Derived source peg for the moving disk at each step. Feeds Sheet2 Status and Keyframes.</t>
         </r>
       </text>
     </comment>
-    <comment ref="E18" authorId="0" shapeId="0" xr:uid="{242B9B47-8033-9044-92CB-22DFD00ACA15}">
+    <comment ref="E19" authorId="0" shapeId="0" xr:uid="{9A33C3E0-5B07-EB45-8AF7-72A9E06E5FBA}">
       <text>
         <r>
           <rPr>
@@ -670,7 +727,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D19" authorId="0" shapeId="0" xr:uid="{600C42A8-8DDE-F946-A285-12B72DF5D886}">
+    <comment ref="D20" authorId="0" shapeId="0" xr:uid="{797C3C03-778E-2045-AF05-43087C4B8149}">
       <text>
         <r>
           <rPr>
@@ -694,7 +751,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E19" authorId="0" shapeId="0" xr:uid="{9A33C3E0-5B07-EB45-8AF7-72A9E06E5FBA}">
+    <comment ref="E20" authorId="0" shapeId="0" xr:uid="{0A4BCC7D-E154-0347-870F-4602B824015B}">
       <text>
         <r>
           <rPr>
@@ -718,7 +775,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D20" authorId="0" shapeId="0" xr:uid="{797C3C03-778E-2045-AF05-43087C4B8149}">
+    <comment ref="D21" authorId="0" shapeId="0" xr:uid="{B6BB8625-CE4D-BA49-8ED6-900492E8E8FE}">
       <text>
         <r>
           <rPr>
@@ -742,7 +799,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E20" authorId="0" shapeId="0" xr:uid="{0A4BCC7D-E154-0347-870F-4602B824015B}">
+    <comment ref="E21" authorId="0" shapeId="0" xr:uid="{69DFDD62-4468-EF41-9D97-5658119195F4}">
       <text>
         <r>
           <rPr>
@@ -766,7 +823,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D21" authorId="0" shapeId="0" xr:uid="{B6BB8625-CE4D-BA49-8ED6-900492E8E8FE}">
+    <comment ref="D22" authorId="0" shapeId="0" xr:uid="{C2D58146-FEC1-2647-B1A0-C818B1C8AF2D}">
       <text>
         <r>
           <rPr>
@@ -790,7 +847,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E21" authorId="0" shapeId="0" xr:uid="{69DFDD62-4468-EF41-9D97-5658119195F4}">
+    <comment ref="E22" authorId="0" shapeId="0" xr:uid="{83ECB3B3-BDF6-184F-A432-A450D3E33728}">
       <text>
         <r>
           <rPr>
@@ -814,7 +871,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D22" authorId="0" shapeId="0" xr:uid="{C2D58146-FEC1-2647-B1A0-C818B1C8AF2D}">
+    <comment ref="D23" authorId="0" shapeId="0" xr:uid="{4185DE22-41DD-1248-AA6D-055CDD4ECAF2}">
       <text>
         <r>
           <rPr>
@@ -838,7 +895,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E22" authorId="0" shapeId="0" xr:uid="{83ECB3B3-BDF6-184F-A432-A450D3E33728}">
+    <comment ref="E23" authorId="0" shapeId="0" xr:uid="{4DD27315-72E1-5F4A-8CCC-1404F81A11B1}">
       <text>
         <r>
           <rPr>
@@ -862,7 +919,64 @@
         </r>
       </text>
     </comment>
-    <comment ref="D23" authorId="0" shapeId="0" xr:uid="{4185DE22-41DD-1248-AA6D-055CDD4ECAF2}">
+    <comment ref="D24" authorId="0" shapeId="0" xr:uid="{3726916B-BB17-0D4D-ADB9-F9FA09FEAAAF}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Yuan Jiang:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Derived source peg for the moving disk at each step. Feeds Sheet2 Status and Keyframes.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E24" authorId="0" shapeId="0" xr:uid="{71D9C3CD-0E91-0641-B1BF-379B6C871062}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Yuan Jiang:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Derived destination peg for the moving disk at each step. Feeds Sheet2 Status and Keyframes.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D25" authorId="0" shapeId="0" xr:uid="{47BB9CD1-7622-C945-AA07-CE034CAA5C6D}">
       <text>
         <r>
           <rPr>
@@ -886,7 +1000,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E23" authorId="0" shapeId="0" xr:uid="{4DD27315-72E1-5F4A-8CCC-1404F81A11B1}">
+    <comment ref="E25" authorId="0" shapeId="0" xr:uid="{C4DBF8DD-E2D0-0B46-8CE3-DAFD62E0E98F}">
       <text>
         <r>
           <rPr>
@@ -910,7 +1024,64 @@
         </r>
       </text>
     </comment>
-    <comment ref="D24" authorId="0" shapeId="0" xr:uid="{3726916B-BB17-0D4D-ADB9-F9FA09FEAAAF}">
+    <comment ref="D26" authorId="0" shapeId="0" xr:uid="{0597B4A6-A773-154D-9827-FE11D3B38D89}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Yuan Jiang:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Derived source peg for the moving disk at each step. Feeds Sheet2 Status and Keyframes.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E26" authorId="0" shapeId="0" xr:uid="{C39FE472-6E95-4846-944E-88DC4A65212B}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Yuan Jiang:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Derived destination peg for the moving disk at each step. Feeds Sheet2 Status and Keyframes.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D27" authorId="0" shapeId="0" xr:uid="{9B06EB71-B963-054C-ADF7-514443B38089}">
       <text>
         <r>
           <rPr>
@@ -934,7 +1105,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E24" authorId="0" shapeId="0" xr:uid="{71D9C3CD-0E91-0641-B1BF-379B6C871062}">
+    <comment ref="E27" authorId="0" shapeId="0" xr:uid="{7A94F625-8ABF-144E-9C6D-63E1681C0365}">
       <text>
         <r>
           <rPr>
@@ -958,7 +1129,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D25" authorId="0" shapeId="0" xr:uid="{47BB9CD1-7622-C945-AA07-CE034CAA5C6D}">
+    <comment ref="D28" authorId="0" shapeId="0" xr:uid="{1E8324D6-1DA1-C24F-9222-AB13541027F1}">
       <text>
         <r>
           <rPr>
@@ -982,7 +1153,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E25" authorId="0" shapeId="0" xr:uid="{C4DBF8DD-E2D0-0B46-8CE3-DAFD62E0E98F}">
+    <comment ref="E28" authorId="0" shapeId="0" xr:uid="{EE5AB279-AC98-5F43-9BED-8532718E3F9D}">
       <text>
         <r>
           <rPr>
@@ -1006,150 +1177,6 @@
         </r>
       </text>
     </comment>
-    <comment ref="D26" authorId="0" shapeId="0" xr:uid="{0597B4A6-A773-154D-9827-FE11D3B38D89}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Yuan Jiang:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Derived source peg for the moving disk at each step. Feeds Sheet2 Status and Keyframes.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E26" authorId="0" shapeId="0" xr:uid="{C39FE472-6E95-4846-944E-88DC4A65212B}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Yuan Jiang:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Derived destination peg for the moving disk at each step. Feeds Sheet2 Status and Keyframes.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D27" authorId="0" shapeId="0" xr:uid="{9B06EB71-B963-054C-ADF7-514443B38089}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Yuan Jiang:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Derived source peg for the moving disk at each step. Feeds Sheet2 Status and Keyframes.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E27" authorId="0" shapeId="0" xr:uid="{7A94F625-8ABF-144E-9C6D-63E1681C0365}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Yuan Jiang:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Derived destination peg for the moving disk at each step. Feeds Sheet2 Status and Keyframes.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D28" authorId="0" shapeId="0" xr:uid="{1E8324D6-1DA1-C24F-9222-AB13541027F1}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Yuan Jiang:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Derived source peg for the moving disk at each step. Feeds Sheet2 Status and Keyframes.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E28" authorId="0" shapeId="0" xr:uid="{EE5AB279-AC98-5F43-9BED-8532718E3F9D}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Yuan Jiang:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Derived destination peg for the moving disk at each step. Feeds Sheet2 Status and Keyframes.</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="D29" authorId="0" shapeId="0" xr:uid="{986ECBB4-20FD-8445-8D59-FFFAECC257FF}">
       <text>
         <r>
@@ -1170,7 +1197,16 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-Derived source peg for the moving disk at each step. Feeds Sheet2 Status and Keyframes.</t>
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Derived source peg for the moving disk at each step. Feeds Sheet2 Status and Keyframes.</t>
         </r>
       </text>
     </comment>
@@ -3381,7 +3417,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -3403,7 +3439,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="49">
   <si>
     <t>│</t>
   </si>
@@ -5620,7 +5656,9 @@
   <we:alternateReferences>
     <we:reference id="wa200010215" version="1.0.0.0" store="WA200010215" storeType="OMEX"/>
   </we:alternateReferences>
-  <we:properties/>
+  <we:properties>
+    <we:property name="bps.codex_control.document_id" value="&quot;36fdf479-3b60-4cf1-817d-474706c33b6c&quot;"/>
+  </we:properties>
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </we:webextension>
@@ -6080,8 +6118,8 @@
       </c>
     </row>
     <row r="6" spans="1:51" ht="26" customHeight="1">
-      <c r="A6" s="89" t="s">
-        <v>4</v>
+      <c r="A6" s="89">
+        <v>3</v>
       </c>
       <c r="B6" s="95">
         <v>0</v>
@@ -6255,7 +6293,9 @@
       <c r="AY6" s="43"/>
     </row>
     <row r="7" spans="1:51" ht="26" customHeight="1" thickBot="1">
-      <c r="A7" s="96"/>
+      <c r="A7" s="96">
+        <v>0</v>
+      </c>
       <c r="B7" s="35"/>
       <c r="C7" s="93"/>
       <c r="D7" s="28" t="str" cm="1">
@@ -6959,7 +6999,7 @@
       </c>
       <c r="B11" s="30" t="str" cm="1">
         <f t="array" ref="B11">HN_PROGRESS_BAR($AY$10,$B$9,10)</f>
-        <v>□□□□□□□□□□  0/10</v>
+        <v>□□□□□□□□□□  0%</v>
       </c>
       <c r="C11" s="93"/>
       <c r="D11" s="28" t="str" cm="1">
@@ -7936,8 +7976,8 @@
       <c r="A5" s="78" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="81">
-        <f>Stage!B5</f>
+      <c r="B5" s="81" cm="1">
+        <f t="array" ref="B5">HN_CLAMP_DISKS(Stage!B5)</f>
         <v>3</v>
       </c>
       <c r="C5" s="84"/>

</xml_diff>

<commit_message>
fix: restore Hanoi stage labels
</commit_message>
<xml_diff>
--- a/Hanoi/Hanoi-1.0.xlsx
+++ b/Hanoi/Hanoi-1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Hanoi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA7E69D7-A897-114E-A520-10216280EA7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36D0E21A-4591-4D48-8603-66D403AF79C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15900" xr2:uid="{82D447F9-66A8-4F40-88AB-946121063596}"/>
   </bookViews>
@@ -3439,7 +3439,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="49">
   <si>
     <t>│</t>
   </si>
@@ -6118,8 +6118,8 @@
       </c>
     </row>
     <row r="6" spans="1:51" ht="26" customHeight="1">
-      <c r="A6" s="89">
-        <v>3</v>
+      <c r="A6" s="89" t="s">
+        <v>4</v>
       </c>
       <c r="B6" s="95">
         <v>0</v>
@@ -6293,9 +6293,7 @@
       <c r="AY6" s="43"/>
     </row>
     <row r="7" spans="1:51" ht="26" customHeight="1" thickBot="1">
-      <c r="A7" s="96">
-        <v>0</v>
-      </c>
+      <c r="A7" s="96"/>
       <c r="B7" s="35"/>
       <c r="C7" s="93"/>
       <c r="D7" s="28" t="str" cm="1">

</xml_diff>

<commit_message>
docs: add Hanoi workbook guide
</commit_message>
<xml_diff>
--- a/Hanoi/Hanoi-1.0.xlsx
+++ b/Hanoi/Hanoi-1.0.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Hanoi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36D0E21A-4591-4D48-8603-66D403AF79C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{919EBE1D-DA9E-F044-B518-DB868D315DCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15900" xr2:uid="{82D447F9-66A8-4F40-88AB-946121063596}"/>
   </bookViews>
   <sheets>
     <sheet name="Stage" sheetId="2" r:id="rId1"/>
-    <sheet name="Engine" sheetId="3" r:id="rId2"/>
+    <sheet name="Guide" sheetId="4" r:id="rId2"/>
+    <sheet name="Engine" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_HanoiActiveAddr">ADDRESS(_HanoiActiveRow,_HanoiActiveCol,4)</definedName>
@@ -3439,7 +3440,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="72">
   <si>
     <t>│</t>
   </si>
@@ -3546,22 +3547,10 @@
     <t>Reserved</t>
   </si>
   <si>
-    <t>Display Mode</t>
-  </si>
-  <si>
-    <t>Full Move</t>
-  </si>
-  <si>
-    <t>Built by ChatGPT · Formula-only Hanoi step demo</t>
-  </si>
-  <si>
     <t>Hanoi Formula Step Demo</t>
   </si>
   <si>
     <t>Active Step List</t>
-  </si>
-  <si>
-    <t>Use B6 to choose the step. If Disks changes, the display clamps to the last valid step until you reselect.</t>
   </si>
   <si>
     <t>Info</t>
@@ -3586,14 +3575,95 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>sleetdrop@gmail.com</t>
+    <t>A formula-only Tower of Hanoi visualizer · Version 1.0.0</t>
+  </si>
+  <si>
+    <t>Quick Start</t>
+  </si>
+  <si>
+    <t>1. Open Stage. Choose 3–6 disks in B5.</t>
+  </si>
+  <si>
+    <t>2. Choose a step in B6 from 0 through Total Steps.</t>
+  </si>
+  <si>
+    <t>3. Follow Current Move, Disk Positions, the Motion Stage, and Keyframes.</t>
+  </si>
+  <si>
+    <t>Formula-Only Boundary</t>
+  </si>
+  <si>
+    <t>No VBA, macros, Office Scripts, custom functions, external runtimes, external data, or external workbook links.</t>
+  </si>
+  <si>
+    <t>Workbook Map</t>
+  </si>
+  <si>
+    <t>Stage — interactive controls, status, motion stage, legend, and keyframes.</t>
+  </si>
+  <si>
+    <t>Guide — usage, architecture, compatibility, and inspection notes.</t>
+  </si>
+  <si>
+    <t>Engine — solved states, active step list, named-formula integration, and release checks.</t>
+  </si>
+  <si>
+    <t>Formula Architecture</t>
+  </si>
+  <si>
+    <t>Stage inputs → HN_CLAMP_DISKS / HN_EFFECTIVE_STEP → Engine solved-state table</t>
+  </si>
+  <si>
+    <t>Engine states → query helpers → Stage title, status, keyframes, and cell-grid rendering</t>
+  </si>
+  <si>
+    <t>Named LAMBDA Groups</t>
+  </si>
+  <si>
+    <t>Input constraints — HN_CLAMP_DISKS, HN_EFFECTIVE_STEP, HN_MAX_STEP</t>
+  </si>
+  <si>
+    <t>Solver logic — HN_MOVE_DISK, HN_DISK_POS, HN_MOVE_ENDPOINT, HN_STEP_LIST</t>
+  </si>
+  <si>
+    <t>Lookup helpers — HN_MOVE_DISK_AT, HN_MOVE_FROM, HN_MOVE_TO, HN_POS_ROW</t>
+  </si>
+  <si>
+    <t>Display helpers — HN_STAGE_CELL, HN_STAGE_TITLE, HN_MOVE_LABEL, HN_PROGRESS_BAR, HN_POSITIONS</t>
+  </si>
+  <si>
+    <t>Compatibility</t>
+  </si>
+  <si>
+    <t>Verified on Microsoft Excel 365 Desktop. Excel 2024 and Excel for Web are unverified.</t>
+  </si>
+  <si>
+    <t>Inspect and Contribute</t>
+  </si>
+  <si>
+    <t>Inspect Engine and Excel Name Manager for the implementation. Report problems through GitHub Issues.</t>
+  </si>
+  <si>
+    <t>Created by Yuan Jiang with ChatGPT as an experiment in formula-only interactive software.</t>
+  </si>
+  <si>
+    <t>Input Status</t>
+  </si>
+  <si>
+    <t>See Guide for instructions. Pasted invalid values are adjusted for display.</t>
+  </si>
+  <si>
+    <t>Guide → see the Guide sheet for usage and formula architecture</t>
+  </si>
+  <si>
+    <t>v1.0.0 · Created by Yuan Jiang with ChatGPT · Formula-only</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18">
+  <fonts count="21">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -3713,6 +3783,25 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10.5"/>
+      <color rgb="FF232A32"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
+      <color rgb="FF215E37"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10.5"/>
+      <color rgb="FF548235"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="12">
     <fill>
@@ -3782,7 +3871,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="97">
+  <borders count="98">
     <border>
       <left/>
       <right/>
@@ -4920,13 +5009,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF548235"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="124">
+  <cellXfs count="130">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -5298,6 +5396,24 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="96" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="97" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5708,7 +5824,7 @@
   <sheetData>
     <row r="1" spans="1:51" ht="26" customHeight="1" thickBot="1">
       <c r="A1" s="25" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
@@ -5763,7 +5879,7 @@
     </row>
     <row r="2" spans="1:51" ht="20" customHeight="1" thickTop="1">
       <c r="A2" s="7" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="7"/>
@@ -7349,17 +7465,18 @@
     </row>
     <row r="13" spans="1:51" ht="24" customHeight="1" thickBot="1">
       <c r="A13" s="92" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="31" t="s">
-        <v>36</v>
+        <v>68</v>
+      </c>
+      <c r="B13" s="31" t="str" cm="1">
+        <f t="array" ref="B13">_xlfn.LET(_xlpm.d,HN_CLAMP_DISKS($B$5),_xlpm.s,HN_EFFECTIVE_STEP($B$6,HN_MAX_STEP(_xlpm.d)),IF(AND($B$5=_xlpm.d,$B$6=_xlpm.s),"Inputs valid","Display adjusted to "&amp;_xlpm.d&amp;" disks / step "&amp;_xlpm.s))</f>
+        <v>Inputs valid</v>
       </c>
       <c r="C13" s="93"/>
       <c r="D13" s="120" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E13" s="122" t="s">
-        <v>40</v>
+        <v>69</v>
       </c>
       <c r="F13" s="122"/>
       <c r="G13" s="122"/>
@@ -7750,7 +7867,7 @@
       <c r="T19" s="35"/>
       <c r="U19" s="35"/>
       <c r="V19" s="121" t="s">
-        <v>48</v>
+        <v>70</v>
       </c>
       <c r="W19" s="35"/>
       <c r="X19" s="35"/>
@@ -7802,7 +7919,7 @@
       <c r="T20" s="93"/>
       <c r="U20" s="93"/>
       <c r="V20" s="110" t="s">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="W20" s="35"/>
       <c r="X20" s="35"/>
@@ -7874,6 +7991,420 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0009E4A1-BE72-1440-A19F-7A09E42F88E2}">
+  <sheetPr>
+    <tabColor rgb="FF548235"/>
+  </sheetPr>
+  <dimension ref="A1:H32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="1" max="8" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="34" customHeight="1">
+      <c r="A1" s="124" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="124"/>
+      <c r="C1" s="124"/>
+      <c r="D1" s="124"/>
+      <c r="E1" s="124"/>
+      <c r="F1" s="124"/>
+      <c r="G1" s="124"/>
+      <c r="H1" s="124"/>
+    </row>
+    <row r="2" spans="1:8" ht="26" customHeight="1">
+      <c r="A2" s="125" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="125"/>
+      <c r="C2" s="125"/>
+      <c r="D2" s="125"/>
+      <c r="E2" s="125"/>
+      <c r="F2" s="125"/>
+      <c r="G2" s="125"/>
+      <c r="H2" s="125"/>
+    </row>
+    <row r="3" spans="1:8" ht="10" customHeight="1">
+      <c r="A3" s="127"/>
+      <c r="B3" s="127"/>
+      <c r="C3" s="127"/>
+      <c r="D3" s="127"/>
+      <c r="E3" s="127"/>
+      <c r="F3" s="127"/>
+      <c r="G3" s="127"/>
+      <c r="H3" s="127"/>
+    </row>
+    <row r="4" spans="1:8" ht="24" customHeight="1">
+      <c r="A4" s="126" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="126"/>
+      <c r="C4" s="126"/>
+      <c r="D4" s="126"/>
+      <c r="E4" s="126"/>
+      <c r="F4" s="126"/>
+      <c r="G4" s="126"/>
+      <c r="H4" s="126"/>
+    </row>
+    <row r="5" spans="1:8" ht="24" customHeight="1">
+      <c r="A5" s="128" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="128"/>
+      <c r="C5" s="128"/>
+      <c r="D5" s="128"/>
+      <c r="E5" s="128"/>
+      <c r="F5" s="128"/>
+      <c r="G5" s="128"/>
+      <c r="H5" s="128"/>
+    </row>
+    <row r="6" spans="1:8" ht="24" customHeight="1">
+      <c r="A6" s="128" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" s="128"/>
+      <c r="C6" s="128"/>
+      <c r="D6" s="128"/>
+      <c r="E6" s="128"/>
+      <c r="F6" s="128"/>
+      <c r="G6" s="128"/>
+      <c r="H6" s="128"/>
+    </row>
+    <row r="7" spans="1:8" ht="30" customHeight="1">
+      <c r="A7" s="128" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="128"/>
+      <c r="C7" s="128"/>
+      <c r="D7" s="128"/>
+      <c r="E7" s="128"/>
+      <c r="F7" s="128"/>
+      <c r="G7" s="128"/>
+      <c r="H7" s="128"/>
+    </row>
+    <row r="8" spans="1:8" ht="10" customHeight="1">
+      <c r="A8" s="127"/>
+      <c r="B8" s="127"/>
+      <c r="C8" s="127"/>
+      <c r="D8" s="127"/>
+      <c r="E8" s="127"/>
+      <c r="F8" s="127"/>
+      <c r="G8" s="127"/>
+      <c r="H8" s="127"/>
+    </row>
+    <row r="9" spans="1:8" ht="24" customHeight="1">
+      <c r="A9" s="126" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" s="126"/>
+      <c r="C9" s="126"/>
+      <c r="D9" s="126"/>
+      <c r="E9" s="126"/>
+      <c r="F9" s="126"/>
+      <c r="G9" s="126"/>
+      <c r="H9" s="126"/>
+    </row>
+    <row r="10" spans="1:8" ht="40" customHeight="1">
+      <c r="A10" s="128" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" s="128"/>
+      <c r="C10" s="128"/>
+      <c r="D10" s="128"/>
+      <c r="E10" s="128"/>
+      <c r="F10" s="128"/>
+      <c r="G10" s="128"/>
+      <c r="H10" s="128"/>
+    </row>
+    <row r="11" spans="1:8" ht="10" customHeight="1">
+      <c r="A11" s="127"/>
+      <c r="B11" s="127"/>
+      <c r="C11" s="127"/>
+      <c r="D11" s="127"/>
+      <c r="E11" s="127"/>
+      <c r="F11" s="127"/>
+      <c r="G11" s="127"/>
+      <c r="H11" s="127"/>
+    </row>
+    <row r="12" spans="1:8" ht="24" customHeight="1">
+      <c r="A12" s="126" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" s="126"/>
+      <c r="C12" s="126"/>
+      <c r="D12" s="126"/>
+      <c r="E12" s="126"/>
+      <c r="F12" s="126"/>
+      <c r="G12" s="126"/>
+      <c r="H12" s="126"/>
+    </row>
+    <row r="13" spans="1:8" ht="26" customHeight="1">
+      <c r="A13" s="128" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" s="128"/>
+      <c r="C13" s="128"/>
+      <c r="D13" s="128"/>
+      <c r="E13" s="128"/>
+      <c r="F13" s="128"/>
+      <c r="G13" s="128"/>
+      <c r="H13" s="128"/>
+    </row>
+    <row r="14" spans="1:8" ht="24" customHeight="1">
+      <c r="A14" s="128" t="s">
+        <v>53</v>
+      </c>
+      <c r="B14" s="128"/>
+      <c r="C14" s="128"/>
+      <c r="D14" s="128"/>
+      <c r="E14" s="128"/>
+      <c r="F14" s="128"/>
+      <c r="G14" s="128"/>
+      <c r="H14" s="128"/>
+    </row>
+    <row r="15" spans="1:8" ht="30" customHeight="1">
+      <c r="A15" s="128" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" s="128"/>
+      <c r="C15" s="128"/>
+      <c r="D15" s="128"/>
+      <c r="E15" s="128"/>
+      <c r="F15" s="128"/>
+      <c r="G15" s="128"/>
+      <c r="H15" s="128"/>
+    </row>
+    <row r="16" spans="1:8" ht="10" customHeight="1">
+      <c r="A16" s="127"/>
+      <c r="B16" s="127"/>
+      <c r="C16" s="127"/>
+      <c r="D16" s="127"/>
+      <c r="E16" s="127"/>
+      <c r="F16" s="127"/>
+      <c r="G16" s="127"/>
+      <c r="H16" s="127"/>
+    </row>
+    <row r="17" spans="1:8" ht="24" customHeight="1">
+      <c r="A17" s="126" t="s">
+        <v>55</v>
+      </c>
+      <c r="B17" s="126"/>
+      <c r="C17" s="126"/>
+      <c r="D17" s="126"/>
+      <c r="E17" s="126"/>
+      <c r="F17" s="126"/>
+      <c r="G17" s="126"/>
+      <c r="H17" s="126"/>
+    </row>
+    <row r="18" spans="1:8" ht="28" customHeight="1">
+      <c r="A18" s="128" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18" s="128"/>
+      <c r="C18" s="128"/>
+      <c r="D18" s="128"/>
+      <c r="E18" s="128"/>
+      <c r="F18" s="128"/>
+      <c r="G18" s="128"/>
+      <c r="H18" s="128"/>
+    </row>
+    <row r="19" spans="1:8" ht="30" customHeight="1">
+      <c r="A19" s="128" t="s">
+        <v>57</v>
+      </c>
+      <c r="B19" s="128"/>
+      <c r="C19" s="128"/>
+      <c r="D19" s="128"/>
+      <c r="E19" s="128"/>
+      <c r="F19" s="128"/>
+      <c r="G19" s="128"/>
+      <c r="H19" s="128"/>
+    </row>
+    <row r="20" spans="1:8" ht="10" customHeight="1">
+      <c r="A20" s="127"/>
+      <c r="B20" s="127"/>
+      <c r="C20" s="127"/>
+      <c r="D20" s="127"/>
+      <c r="E20" s="127"/>
+      <c r="F20" s="127"/>
+      <c r="G20" s="127"/>
+      <c r="H20" s="127"/>
+    </row>
+    <row r="21" spans="1:8" ht="24" customHeight="1">
+      <c r="A21" s="126" t="s">
+        <v>58</v>
+      </c>
+      <c r="B21" s="126"/>
+      <c r="C21" s="126"/>
+      <c r="D21" s="126"/>
+      <c r="E21" s="126"/>
+      <c r="F21" s="126"/>
+      <c r="G21" s="126"/>
+      <c r="H21" s="126"/>
+    </row>
+    <row r="22" spans="1:8" ht="26" customHeight="1">
+      <c r="A22" s="128" t="s">
+        <v>59</v>
+      </c>
+      <c r="B22" s="128"/>
+      <c r="C22" s="128"/>
+      <c r="D22" s="128"/>
+      <c r="E22" s="128"/>
+      <c r="F22" s="128"/>
+      <c r="G22" s="128"/>
+      <c r="H22" s="128"/>
+    </row>
+    <row r="23" spans="1:8" ht="28" customHeight="1">
+      <c r="A23" s="128" t="s">
+        <v>60</v>
+      </c>
+      <c r="B23" s="128"/>
+      <c r="C23" s="128"/>
+      <c r="D23" s="128"/>
+      <c r="E23" s="128"/>
+      <c r="F23" s="128"/>
+      <c r="G23" s="128"/>
+      <c r="H23" s="128"/>
+    </row>
+    <row r="24" spans="1:8" ht="26" customHeight="1">
+      <c r="A24" s="128" t="s">
+        <v>61</v>
+      </c>
+      <c r="B24" s="128"/>
+      <c r="C24" s="128"/>
+      <c r="D24" s="128"/>
+      <c r="E24" s="128"/>
+      <c r="F24" s="128"/>
+      <c r="G24" s="128"/>
+      <c r="H24" s="128"/>
+    </row>
+    <row r="25" spans="1:8" ht="36" customHeight="1">
+      <c r="A25" s="128" t="s">
+        <v>62</v>
+      </c>
+      <c r="B25" s="128"/>
+      <c r="C25" s="128"/>
+      <c r="D25" s="128"/>
+      <c r="E25" s="128"/>
+      <c r="F25" s="128"/>
+      <c r="G25" s="128"/>
+      <c r="H25" s="128"/>
+    </row>
+    <row r="26" spans="1:8" ht="10" customHeight="1">
+      <c r="A26" s="127"/>
+      <c r="B26" s="127"/>
+      <c r="C26" s="127"/>
+      <c r="D26" s="127"/>
+      <c r="E26" s="127"/>
+      <c r="F26" s="127"/>
+      <c r="G26" s="127"/>
+      <c r="H26" s="127"/>
+    </row>
+    <row r="27" spans="1:8" ht="24" customHeight="1">
+      <c r="A27" s="126" t="s">
+        <v>63</v>
+      </c>
+      <c r="B27" s="126"/>
+      <c r="C27" s="126"/>
+      <c r="D27" s="126"/>
+      <c r="E27" s="126"/>
+      <c r="F27" s="126"/>
+      <c r="G27" s="126"/>
+      <c r="H27" s="126"/>
+    </row>
+    <row r="28" spans="1:8" ht="30" customHeight="1">
+      <c r="A28" s="128" t="s">
+        <v>64</v>
+      </c>
+      <c r="B28" s="128"/>
+      <c r="C28" s="128"/>
+      <c r="D28" s="128"/>
+      <c r="E28" s="128"/>
+      <c r="F28" s="128"/>
+      <c r="G28" s="128"/>
+      <c r="H28" s="128"/>
+    </row>
+    <row r="29" spans="1:8" ht="10" customHeight="1">
+      <c r="A29" s="127"/>
+      <c r="B29" s="127"/>
+      <c r="C29" s="127"/>
+      <c r="D29" s="127"/>
+      <c r="E29" s="127"/>
+      <c r="F29" s="127"/>
+      <c r="G29" s="127"/>
+      <c r="H29" s="127"/>
+    </row>
+    <row r="30" spans="1:8" ht="24" customHeight="1">
+      <c r="A30" s="126" t="s">
+        <v>65</v>
+      </c>
+      <c r="B30" s="126"/>
+      <c r="C30" s="126"/>
+      <c r="D30" s="126"/>
+      <c r="E30" s="126"/>
+      <c r="F30" s="126"/>
+      <c r="G30" s="126"/>
+      <c r="H30" s="126"/>
+    </row>
+    <row r="31" spans="1:8" ht="34" customHeight="1">
+      <c r="A31" s="128" t="s">
+        <v>66</v>
+      </c>
+      <c r="B31" s="128"/>
+      <c r="C31" s="128"/>
+      <c r="D31" s="128"/>
+      <c r="E31" s="128"/>
+      <c r="F31" s="128"/>
+      <c r="G31" s="128"/>
+      <c r="H31" s="128"/>
+    </row>
+    <row r="32" spans="1:8" ht="30" customHeight="1">
+      <c r="A32" s="129" t="s">
+        <v>67</v>
+      </c>
+      <c r="B32" s="129"/>
+      <c r="C32" s="129"/>
+      <c r="D32" s="129"/>
+      <c r="E32" s="129"/>
+      <c r="F32" s="129"/>
+      <c r="G32" s="129"/>
+      <c r="H32" s="129"/>
+    </row>
+  </sheetData>
+  <mergeCells count="25">
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A7:H7"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4B11188-EA99-1948-A4A2-27BFA73FC50E}">
   <sheetPr>
     <tabColor rgb="FF70AD47"/>
@@ -7907,12 +8438,12 @@
       <c r="K1" s="4"/>
       <c r="L1" s="115"/>
       <c r="M1" s="68" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="17" thickTop="1">
       <c r="A2" s="6" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="7"/>
@@ -7932,7 +8463,7 @@
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="9" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B3" s="10"/>
       <c r="C3" s="10"/>
@@ -7980,7 +8511,7 @@
       </c>
       <c r="C5" s="84"/>
       <c r="D5" s="74" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="E5" s="69"/>
       <c r="F5" s="69"/>
@@ -8004,7 +8535,7 @@
       </c>
       <c r="C6" s="84"/>
       <c r="D6" s="17" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E6" s="18"/>
       <c r="F6" s="18"/>
@@ -8028,7 +8559,7 @@
       </c>
       <c r="C7" s="84"/>
       <c r="D7" s="75" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="E7" s="73"/>
       <c r="F7" s="73"/>

</xml_diff>

<commit_message>
chore: sanitize Hanoi workbook package
</commit_message>
<xml_diff>
--- a/Hanoi/Hanoi-1.0.xlsx
+++ b/Hanoi/Hanoi-1.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Hanoi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E786604B-2916-5E49-9DC8-7BAA4506F5AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8614F1C1-E031-414D-9764-50EEF05ACB3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15820" xr2:uid="{82D447F9-66A8-4F40-88AB-946121063596}"/>
+    <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15840" xr2:uid="{82D447F9-66A8-4F40-88AB-946121063596}"/>
   </bookViews>
   <sheets>
     <sheet name="Stage" sheetId="2" r:id="rId1"/>
@@ -18,9 +18,6 @@
     <sheet name="Engine" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_HanoiActiveAddr">ADDRESS(_HanoiActiveRow,_HanoiActiveCol,4)</definedName>
-    <definedName name="_HanoiActiveCol">COLUMN(_HanoiActiveCell)</definedName>
-    <definedName name="_HanoiActiveRow">ROW(_HanoiActiveCell)</definedName>
     <definedName name="_HanoiStepList">_xlfn.ANCHORARRAY(Engine!$M$2)</definedName>
     <definedName name="HanoiDisks">Stage!$B$5</definedName>
     <definedName name="HanoiMaxStep">Engine!$B$6</definedName>
@@ -68,7 +65,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -2038,6 +2035,27 @@
     <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2058,27 +2076,6 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2431,53 +2428,6 @@
 </a:theme>
 </file>
 
-<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
-<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </wetp:taskpane>
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-  </wetp:taskpane>
-</wetp:taskpanes>
-</file>
-
-<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{ADC4393F-D646-454A-8E02-70262B39FB86}">
-  <we:reference id="wa200010215" version="1.0.0.0" store="en-US" storeType="OMEX"/>
-  <we:alternateReferences>
-    <we:reference id="wa200010215" version="1.0.0.0" store="WA200010215" storeType="OMEX"/>
-  </we:alternateReferences>
-  <we:properties>
-    <we:property name="bps.codex_control.document_id" value="&quot;36fdf479-3b60-4cf1-817d-474706c33b6c&quot;"/>
-  </we:properties>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</we:webextension>
-</file>
-
-<file path=xl/webextensions/webextension2.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{9AE83F60-0D61-8844-BBF4-C420236ED2C7}">
-  <we:reference id="wa200003696" version="1.3.0.0" store="en-US" storeType="OMEX"/>
-  <we:alternateReferences>
-    <we:reference id="WA200003696" version="1.3.0.0" store="" storeType="OMEX"/>
-  </we:alternateReferences>
-  <we:properties/>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-  <we:extLst>
-    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
-      <we:containsCustomFunctions/>
-    </a:ext>
-    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
-      <we:customFunctionIdList>
-        <we:customFunctionIds>_xldudf_LABS_GENERATIVEAI</we:customFunctionIds>
-      </we:customFunctionIdList>
-    </a:ext>
-  </we:extLst>
-</we:webextension>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{808EFA45-B4F0-2A4C-B273-D330143269CF}">
   <sheetPr>
@@ -4151,44 +4101,44 @@
       <c r="D13" s="119" t="s">
         <v>36</v>
       </c>
-      <c r="E13" s="122" t="s">
+      <c r="E13" s="129" t="s">
         <v>63</v>
       </c>
-      <c r="F13" s="122"/>
-      <c r="G13" s="122"/>
-      <c r="H13" s="122"/>
-      <c r="I13" s="122"/>
-      <c r="J13" s="122"/>
-      <c r="K13" s="122"/>
-      <c r="L13" s="122"/>
-      <c r="M13" s="122"/>
-      <c r="N13" s="122"/>
-      <c r="O13" s="122"/>
-      <c r="P13" s="122"/>
-      <c r="Q13" s="122"/>
-      <c r="R13" s="122"/>
-      <c r="S13" s="122"/>
-      <c r="T13" s="122"/>
-      <c r="U13" s="122"/>
-      <c r="V13" s="122"/>
-      <c r="W13" s="122"/>
-      <c r="X13" s="122"/>
-      <c r="Y13" s="122"/>
-      <c r="Z13" s="122"/>
-      <c r="AA13" s="122"/>
-      <c r="AB13" s="122"/>
-      <c r="AC13" s="122"/>
-      <c r="AD13" s="122"/>
-      <c r="AE13" s="122"/>
-      <c r="AF13" s="122"/>
-      <c r="AG13" s="122"/>
-      <c r="AH13" s="122"/>
-      <c r="AI13" s="122"/>
-      <c r="AJ13" s="122"/>
-      <c r="AK13" s="122"/>
-      <c r="AL13" s="122"/>
-      <c r="AM13" s="122"/>
-      <c r="AN13" s="123"/>
+      <c r="F13" s="129"/>
+      <c r="G13" s="129"/>
+      <c r="H13" s="129"/>
+      <c r="I13" s="129"/>
+      <c r="J13" s="129"/>
+      <c r="K13" s="129"/>
+      <c r="L13" s="129"/>
+      <c r="M13" s="129"/>
+      <c r="N13" s="129"/>
+      <c r="O13" s="129"/>
+      <c r="P13" s="129"/>
+      <c r="Q13" s="129"/>
+      <c r="R13" s="129"/>
+      <c r="S13" s="129"/>
+      <c r="T13" s="129"/>
+      <c r="U13" s="129"/>
+      <c r="V13" s="129"/>
+      <c r="W13" s="129"/>
+      <c r="X13" s="129"/>
+      <c r="Y13" s="129"/>
+      <c r="Z13" s="129"/>
+      <c r="AA13" s="129"/>
+      <c r="AB13" s="129"/>
+      <c r="AC13" s="129"/>
+      <c r="AD13" s="129"/>
+      <c r="AE13" s="129"/>
+      <c r="AF13" s="129"/>
+      <c r="AG13" s="129"/>
+      <c r="AH13" s="129"/>
+      <c r="AI13" s="129"/>
+      <c r="AJ13" s="129"/>
+      <c r="AK13" s="129"/>
+      <c r="AL13" s="129"/>
+      <c r="AM13" s="129"/>
+      <c r="AN13" s="130"/>
       <c r="AO13" s="34"/>
       <c r="AP13" s="112" cm="1">
         <f t="array" ref="AP13">HN_KEYFRAME_STEP($AY$10,HN_MAX_STEP(HN_CLAMP_DISKS($B$5)),ROW()-11)</f>
@@ -4677,28 +4627,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="34" customHeight="1">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="134" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="127"/>
-      <c r="C1" s="127"/>
-      <c r="D1" s="127"/>
-      <c r="E1" s="127"/>
-      <c r="F1" s="127"/>
-      <c r="G1" s="127"/>
-      <c r="H1" s="127"/>
+      <c r="B1" s="134"/>
+      <c r="C1" s="134"/>
+      <c r="D1" s="134"/>
+      <c r="E1" s="134"/>
+      <c r="F1" s="134"/>
+      <c r="G1" s="134"/>
+      <c r="H1" s="134"/>
     </row>
     <row r="2" spans="1:8" ht="26" customHeight="1">
-      <c r="A2" s="128" t="s">
+      <c r="A2" s="135" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="128"/>
-      <c r="C2" s="128"/>
-      <c r="D2" s="128"/>
-      <c r="E2" s="128"/>
-      <c r="F2" s="128"/>
-      <c r="G2" s="128"/>
-      <c r="H2" s="128"/>
+      <c r="B2" s="135"/>
+      <c r="C2" s="135"/>
+      <c r="D2" s="135"/>
+      <c r="E2" s="135"/>
+      <c r="F2" s="135"/>
+      <c r="G2" s="135"/>
+      <c r="H2" s="135"/>
     </row>
     <row r="3" spans="1:8" ht="10" customHeight="1">
       <c r="A3" s="121"/>
@@ -4711,52 +4661,52 @@
       <c r="H3" s="121"/>
     </row>
     <row r="4" spans="1:8" ht="24" customHeight="1">
-      <c r="A4" s="126" t="s">
+      <c r="A4" s="133" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="126"/>
-      <c r="C4" s="126"/>
-      <c r="D4" s="126"/>
-      <c r="E4" s="126"/>
-      <c r="F4" s="126"/>
-      <c r="G4" s="126"/>
-      <c r="H4" s="126"/>
+      <c r="B4" s="133"/>
+      <c r="C4" s="133"/>
+      <c r="D4" s="133"/>
+      <c r="E4" s="133"/>
+      <c r="F4" s="133"/>
+      <c r="G4" s="133"/>
+      <c r="H4" s="133"/>
     </row>
     <row r="5" spans="1:8" ht="24" customHeight="1">
-      <c r="A5" s="125" t="s">
+      <c r="A5" s="132" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="125"/>
-      <c r="C5" s="125"/>
-      <c r="D5" s="125"/>
-      <c r="E5" s="125"/>
-      <c r="F5" s="125"/>
-      <c r="G5" s="125"/>
-      <c r="H5" s="125"/>
+      <c r="B5" s="132"/>
+      <c r="C5" s="132"/>
+      <c r="D5" s="132"/>
+      <c r="E5" s="132"/>
+      <c r="F5" s="132"/>
+      <c r="G5" s="132"/>
+      <c r="H5" s="132"/>
     </row>
     <row r="6" spans="1:8" ht="24" customHeight="1">
-      <c r="A6" s="125" t="s">
+      <c r="A6" s="132" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="125"/>
-      <c r="C6" s="125"/>
-      <c r="D6" s="125"/>
-      <c r="E6" s="125"/>
-      <c r="F6" s="125"/>
-      <c r="G6" s="125"/>
-      <c r="H6" s="125"/>
+      <c r="B6" s="132"/>
+      <c r="C6" s="132"/>
+      <c r="D6" s="132"/>
+      <c r="E6" s="132"/>
+      <c r="F6" s="132"/>
+      <c r="G6" s="132"/>
+      <c r="H6" s="132"/>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1">
-      <c r="A7" s="125" t="s">
+      <c r="A7" s="132" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="125"/>
-      <c r="C7" s="125"/>
-      <c r="D7" s="125"/>
-      <c r="E7" s="125"/>
-      <c r="F7" s="125"/>
-      <c r="G7" s="125"/>
-      <c r="H7" s="125"/>
+      <c r="B7" s="132"/>
+      <c r="C7" s="132"/>
+      <c r="D7" s="132"/>
+      <c r="E7" s="132"/>
+      <c r="F7" s="132"/>
+      <c r="G7" s="132"/>
+      <c r="H7" s="132"/>
     </row>
     <row r="8" spans="1:8" ht="10" customHeight="1">
       <c r="A8" s="121"/>
@@ -4769,28 +4719,28 @@
       <c r="H8" s="121"/>
     </row>
     <row r="9" spans="1:8" ht="24" customHeight="1">
-      <c r="A9" s="126" t="s">
+      <c r="A9" s="133" t="s">
         <v>43</v>
       </c>
-      <c r="B9" s="126"/>
-      <c r="C9" s="126"/>
-      <c r="D9" s="126"/>
-      <c r="E9" s="126"/>
-      <c r="F9" s="126"/>
-      <c r="G9" s="126"/>
-      <c r="H9" s="126"/>
+      <c r="B9" s="133"/>
+      <c r="C9" s="133"/>
+      <c r="D9" s="133"/>
+      <c r="E9" s="133"/>
+      <c r="F9" s="133"/>
+      <c r="G9" s="133"/>
+      <c r="H9" s="133"/>
     </row>
     <row r="10" spans="1:8" ht="40" customHeight="1">
-      <c r="A10" s="125" t="s">
+      <c r="A10" s="132" t="s">
         <v>44</v>
       </c>
-      <c r="B10" s="125"/>
-      <c r="C10" s="125"/>
-      <c r="D10" s="125"/>
-      <c r="E10" s="125"/>
-      <c r="F10" s="125"/>
-      <c r="G10" s="125"/>
-      <c r="H10" s="125"/>
+      <c r="B10" s="132"/>
+      <c r="C10" s="132"/>
+      <c r="D10" s="132"/>
+      <c r="E10" s="132"/>
+      <c r="F10" s="132"/>
+      <c r="G10" s="132"/>
+      <c r="H10" s="132"/>
     </row>
     <row r="11" spans="1:8" ht="10" customHeight="1">
       <c r="A11" s="121"/>
@@ -4803,52 +4753,52 @@
       <c r="H11" s="121"/>
     </row>
     <row r="12" spans="1:8" ht="24" customHeight="1">
-      <c r="A12" s="126" t="s">
+      <c r="A12" s="133" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="126"/>
-      <c r="C12" s="126"/>
-      <c r="D12" s="126"/>
-      <c r="E12" s="126"/>
-      <c r="F12" s="126"/>
-      <c r="G12" s="126"/>
-      <c r="H12" s="126"/>
+      <c r="B12" s="133"/>
+      <c r="C12" s="133"/>
+      <c r="D12" s="133"/>
+      <c r="E12" s="133"/>
+      <c r="F12" s="133"/>
+      <c r="G12" s="133"/>
+      <c r="H12" s="133"/>
     </row>
     <row r="13" spans="1:8" ht="26" customHeight="1">
-      <c r="A13" s="125" t="s">
+      <c r="A13" s="132" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="125"/>
-      <c r="C13" s="125"/>
-      <c r="D13" s="125"/>
-      <c r="E13" s="125"/>
-      <c r="F13" s="125"/>
-      <c r="G13" s="125"/>
-      <c r="H13" s="125"/>
+      <c r="B13" s="132"/>
+      <c r="C13" s="132"/>
+      <c r="D13" s="132"/>
+      <c r="E13" s="132"/>
+      <c r="F13" s="132"/>
+      <c r="G13" s="132"/>
+      <c r="H13" s="132"/>
     </row>
     <row r="14" spans="1:8" ht="24" customHeight="1">
-      <c r="A14" s="125" t="s">
+      <c r="A14" s="132" t="s">
         <v>47</v>
       </c>
-      <c r="B14" s="125"/>
-      <c r="C14" s="125"/>
-      <c r="D14" s="125"/>
-      <c r="E14" s="125"/>
-      <c r="F14" s="125"/>
-      <c r="G14" s="125"/>
-      <c r="H14" s="125"/>
+      <c r="B14" s="132"/>
+      <c r="C14" s="132"/>
+      <c r="D14" s="132"/>
+      <c r="E14" s="132"/>
+      <c r="F14" s="132"/>
+      <c r="G14" s="132"/>
+      <c r="H14" s="132"/>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1">
-      <c r="A15" s="125" t="s">
+      <c r="A15" s="132" t="s">
         <v>48</v>
       </c>
-      <c r="B15" s="125"/>
-      <c r="C15" s="125"/>
-      <c r="D15" s="125"/>
-      <c r="E15" s="125"/>
-      <c r="F15" s="125"/>
-      <c r="G15" s="125"/>
-      <c r="H15" s="125"/>
+      <c r="B15" s="132"/>
+      <c r="C15" s="132"/>
+      <c r="D15" s="132"/>
+      <c r="E15" s="132"/>
+      <c r="F15" s="132"/>
+      <c r="G15" s="132"/>
+      <c r="H15" s="132"/>
     </row>
     <row r="16" spans="1:8" ht="10" customHeight="1">
       <c r="A16" s="121"/>
@@ -4861,40 +4811,40 @@
       <c r="H16" s="121"/>
     </row>
     <row r="17" spans="1:8" ht="24" customHeight="1">
-      <c r="A17" s="126" t="s">
+      <c r="A17" s="133" t="s">
         <v>49</v>
       </c>
-      <c r="B17" s="126"/>
-      <c r="C17" s="126"/>
-      <c r="D17" s="126"/>
-      <c r="E17" s="126"/>
-      <c r="F17" s="126"/>
-      <c r="G17" s="126"/>
-      <c r="H17" s="126"/>
+      <c r="B17" s="133"/>
+      <c r="C17" s="133"/>
+      <c r="D17" s="133"/>
+      <c r="E17" s="133"/>
+      <c r="F17" s="133"/>
+      <c r="G17" s="133"/>
+      <c r="H17" s="133"/>
     </row>
     <row r="18" spans="1:8" ht="28" customHeight="1">
-      <c r="A18" s="125" t="s">
+      <c r="A18" s="132" t="s">
         <v>50</v>
       </c>
-      <c r="B18" s="125"/>
-      <c r="C18" s="125"/>
-      <c r="D18" s="125"/>
-      <c r="E18" s="125"/>
-      <c r="F18" s="125"/>
-      <c r="G18" s="125"/>
-      <c r="H18" s="125"/>
+      <c r="B18" s="132"/>
+      <c r="C18" s="132"/>
+      <c r="D18" s="132"/>
+      <c r="E18" s="132"/>
+      <c r="F18" s="132"/>
+      <c r="G18" s="132"/>
+      <c r="H18" s="132"/>
     </row>
     <row r="19" spans="1:8" ht="30" customHeight="1">
-      <c r="A19" s="125" t="s">
+      <c r="A19" s="132" t="s">
         <v>51</v>
       </c>
-      <c r="B19" s="125"/>
-      <c r="C19" s="125"/>
-      <c r="D19" s="125"/>
-      <c r="E19" s="125"/>
-      <c r="F19" s="125"/>
-      <c r="G19" s="125"/>
-      <c r="H19" s="125"/>
+      <c r="B19" s="132"/>
+      <c r="C19" s="132"/>
+      <c r="D19" s="132"/>
+      <c r="E19" s="132"/>
+      <c r="F19" s="132"/>
+      <c r="G19" s="132"/>
+      <c r="H19" s="132"/>
     </row>
     <row r="20" spans="1:8" ht="10" customHeight="1">
       <c r="A20" s="121"/>
@@ -4907,64 +4857,64 @@
       <c r="H20" s="121"/>
     </row>
     <row r="21" spans="1:8" ht="24" customHeight="1">
-      <c r="A21" s="126" t="s">
+      <c r="A21" s="133" t="s">
         <v>52</v>
       </c>
-      <c r="B21" s="126"/>
-      <c r="C21" s="126"/>
-      <c r="D21" s="126"/>
-      <c r="E21" s="126"/>
-      <c r="F21" s="126"/>
-      <c r="G21" s="126"/>
-      <c r="H21" s="126"/>
+      <c r="B21" s="133"/>
+      <c r="C21" s="133"/>
+      <c r="D21" s="133"/>
+      <c r="E21" s="133"/>
+      <c r="F21" s="133"/>
+      <c r="G21" s="133"/>
+      <c r="H21" s="133"/>
     </row>
     <row r="22" spans="1:8" ht="26" customHeight="1">
-      <c r="A22" s="125" t="s">
+      <c r="A22" s="132" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="125"/>
-      <c r="C22" s="125"/>
-      <c r="D22" s="125"/>
-      <c r="E22" s="125"/>
-      <c r="F22" s="125"/>
-      <c r="G22" s="125"/>
-      <c r="H22" s="125"/>
+      <c r="B22" s="132"/>
+      <c r="C22" s="132"/>
+      <c r="D22" s="132"/>
+      <c r="E22" s="132"/>
+      <c r="F22" s="132"/>
+      <c r="G22" s="132"/>
+      <c r="H22" s="132"/>
     </row>
     <row r="23" spans="1:8" ht="28" customHeight="1">
-      <c r="A23" s="125" t="s">
+      <c r="A23" s="132" t="s">
         <v>54</v>
       </c>
-      <c r="B23" s="125"/>
-      <c r="C23" s="125"/>
-      <c r="D23" s="125"/>
-      <c r="E23" s="125"/>
-      <c r="F23" s="125"/>
-      <c r="G23" s="125"/>
-      <c r="H23" s="125"/>
+      <c r="B23" s="132"/>
+      <c r="C23" s="132"/>
+      <c r="D23" s="132"/>
+      <c r="E23" s="132"/>
+      <c r="F23" s="132"/>
+      <c r="G23" s="132"/>
+      <c r="H23" s="132"/>
     </row>
     <row r="24" spans="1:8" ht="26" customHeight="1">
-      <c r="A24" s="125" t="s">
+      <c r="A24" s="132" t="s">
         <v>55</v>
       </c>
-      <c r="B24" s="125"/>
-      <c r="C24" s="125"/>
-      <c r="D24" s="125"/>
-      <c r="E24" s="125"/>
-      <c r="F24" s="125"/>
-      <c r="G24" s="125"/>
-      <c r="H24" s="125"/>
+      <c r="B24" s="132"/>
+      <c r="C24" s="132"/>
+      <c r="D24" s="132"/>
+      <c r="E24" s="132"/>
+      <c r="F24" s="132"/>
+      <c r="G24" s="132"/>
+      <c r="H24" s="132"/>
     </row>
     <row r="25" spans="1:8" ht="36" customHeight="1">
-      <c r="A25" s="125" t="s">
+      <c r="A25" s="132" t="s">
         <v>56</v>
       </c>
-      <c r="B25" s="125"/>
-      <c r="C25" s="125"/>
-      <c r="D25" s="125"/>
-      <c r="E25" s="125"/>
-      <c r="F25" s="125"/>
-      <c r="G25" s="125"/>
-      <c r="H25" s="125"/>
+      <c r="B25" s="132"/>
+      <c r="C25" s="132"/>
+      <c r="D25" s="132"/>
+      <c r="E25" s="132"/>
+      <c r="F25" s="132"/>
+      <c r="G25" s="132"/>
+      <c r="H25" s="132"/>
     </row>
     <row r="26" spans="1:8" ht="10" customHeight="1">
       <c r="A26" s="121"/>
@@ -4977,28 +4927,28 @@
       <c r="H26" s="121"/>
     </row>
     <row r="27" spans="1:8" ht="24" customHeight="1">
-      <c r="A27" s="126" t="s">
+      <c r="A27" s="133" t="s">
         <v>57</v>
       </c>
-      <c r="B27" s="126"/>
-      <c r="C27" s="126"/>
-      <c r="D27" s="126"/>
-      <c r="E27" s="126"/>
-      <c r="F27" s="126"/>
-      <c r="G27" s="126"/>
-      <c r="H27" s="126"/>
+      <c r="B27" s="133"/>
+      <c r="C27" s="133"/>
+      <c r="D27" s="133"/>
+      <c r="E27" s="133"/>
+      <c r="F27" s="133"/>
+      <c r="G27" s="133"/>
+      <c r="H27" s="133"/>
     </row>
     <row r="28" spans="1:8" ht="30" customHeight="1">
-      <c r="A28" s="125" t="s">
+      <c r="A28" s="132" t="s">
         <v>58</v>
       </c>
-      <c r="B28" s="125"/>
-      <c r="C28" s="125"/>
-      <c r="D28" s="125"/>
-      <c r="E28" s="125"/>
-      <c r="F28" s="125"/>
-      <c r="G28" s="125"/>
-      <c r="H28" s="125"/>
+      <c r="B28" s="132"/>
+      <c r="C28" s="132"/>
+      <c r="D28" s="132"/>
+      <c r="E28" s="132"/>
+      <c r="F28" s="132"/>
+      <c r="G28" s="132"/>
+      <c r="H28" s="132"/>
     </row>
     <row r="29" spans="1:8" ht="10" customHeight="1">
       <c r="A29" s="121"/>
@@ -5011,40 +4961,40 @@
       <c r="H29" s="121"/>
     </row>
     <row r="30" spans="1:8" ht="24" customHeight="1">
-      <c r="A30" s="126" t="s">
+      <c r="A30" s="133" t="s">
         <v>59</v>
       </c>
-      <c r="B30" s="126"/>
-      <c r="C30" s="126"/>
-      <c r="D30" s="126"/>
-      <c r="E30" s="126"/>
-      <c r="F30" s="126"/>
-      <c r="G30" s="126"/>
-      <c r="H30" s="126"/>
+      <c r="B30" s="133"/>
+      <c r="C30" s="133"/>
+      <c r="D30" s="133"/>
+      <c r="E30" s="133"/>
+      <c r="F30" s="133"/>
+      <c r="G30" s="133"/>
+      <c r="H30" s="133"/>
     </row>
     <row r="31" spans="1:8" ht="34" customHeight="1">
-      <c r="A31" s="125" t="s">
+      <c r="A31" s="132" t="s">
         <v>60</v>
       </c>
-      <c r="B31" s="125"/>
-      <c r="C31" s="125"/>
-      <c r="D31" s="125"/>
-      <c r="E31" s="125"/>
-      <c r="F31" s="125"/>
-      <c r="G31" s="125"/>
-      <c r="H31" s="125"/>
+      <c r="B31" s="132"/>
+      <c r="C31" s="132"/>
+      <c r="D31" s="132"/>
+      <c r="E31" s="132"/>
+      <c r="F31" s="132"/>
+      <c r="G31" s="132"/>
+      <c r="H31" s="132"/>
     </row>
     <row r="32" spans="1:8" ht="30" customHeight="1">
-      <c r="A32" s="124" t="s">
+      <c r="A32" s="131" t="s">
         <v>61</v>
       </c>
-      <c r="B32" s="124"/>
-      <c r="C32" s="124"/>
-      <c r="D32" s="124"/>
-      <c r="E32" s="124"/>
-      <c r="F32" s="124"/>
-      <c r="G32" s="124"/>
-      <c r="H32" s="124"/>
+      <c r="B32" s="131"/>
+      <c r="C32" s="131"/>
+      <c r="D32" s="131"/>
+      <c r="E32" s="131"/>
+      <c r="F32" s="131"/>
+      <c r="G32" s="131"/>
+      <c r="H32" s="131"/>
     </row>
   </sheetData>
   <mergeCells count="25">
@@ -5137,7 +5087,7 @@
       </c>
     </row>
     <row r="3" spans="1:13" ht="30">
-      <c r="A3" s="129" t="s">
+      <c r="A3" s="122" t="s">
         <v>67</v>
       </c>
       <c r="B3" s="9"/>
@@ -5164,7 +5114,7 @@
       <c r="D4" s="70" t="s">
         <v>68</v>
       </c>
-      <c r="E4" s="130" t="s">
+      <c r="E4" s="123" t="s">
         <v>69</v>
       </c>
       <c r="F4" s="70"/>
@@ -5190,7 +5140,7 @@
       <c r="D5" s="73" t="s">
         <v>70</v>
       </c>
-      <c r="E5" s="132" t="str">
+      <c r="E5" s="125" t="str">
         <f>IF($B$6=2^$B$5-1,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
@@ -5217,7 +5167,7 @@
       <c r="D6" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="E6" s="133" t="str" cm="1">
+      <c r="E6" s="126" t="str" cm="1">
         <f t="array" ref="E6">_xlfn.LET(_xlpm.n,$B$5,_xlpm.m,$B$6,_xlpm.p,_xlfn.TAKE($F$11:$K$74,_xlpm.m+1,_xlpm.n),_xlpm.c,--(_xlfn.DROP(_xlpm.p,1)&lt;&gt;_xlfn.TAKE(_xlpm.p,_xlpm.m)),IF(AND(_xlfn.BYROW(_xlpm.c,_xlfn.LAMBDA(_xlpm.r,SUM(_xlpm.r)))=1),"PASS","FAIL"))</f>
         <v>PASS</v>
       </c>
@@ -5244,7 +5194,7 @@
       <c r="D7" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="E7" s="134" t="str" cm="1">
+      <c r="E7" s="127" t="str" cm="1">
         <f t="array" ref="E7">_xlfn.LET(_xlpm.m,$B$6,_xlpm.src,_xlfn.TAKE($D$12:$D$74,_xlpm.m),_xlpm.dst,_xlfn.TAKE($E$12:$E$74,_xlpm.m),IF(AND((_xlpm.src&lt;&gt;"")*(_xlpm.dst&lt;&gt;"")*(_xlpm.src&lt;&gt;_xlpm.dst)),"PASS","FAIL"))</f>
         <v>PASS</v>
       </c>
@@ -5263,10 +5213,10 @@
       <c r="A8" s="71"/>
       <c r="B8" s="66"/>
       <c r="C8" s="53"/>
-      <c r="D8" s="131" t="s">
+      <c r="D8" s="124" t="s">
         <v>73</v>
       </c>
-      <c r="E8" s="135" t="str" cm="1">
+      <c r="E8" s="128" t="str" cm="1">
         <f t="array" ref="E8">_xlfn.LET(_xlpm.n,$B$5,_xlpm.m,$B$6,_xlpm.last,_xlfn.XLOOKUP(_xlpm.m,$A$11:$A$74,$F$11:$K$74),IF(AND(_xlfn.TAKE(_xlpm.last,,_xlpm.n)=3),"PASS","FAIL"))</f>
         <v>PASS</v>
       </c>
@@ -5290,7 +5240,7 @@
       <c r="D9" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="E9" s="133" t="str">
+      <c r="E9" s="126" t="str">
         <f>IF(COUNTIF($E$5:$E$8,"PASS")=4,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
@@ -8227,8 +8177,6 @@
     <cfRule type="expression" dxfId="1" priority="1">
       <formula>E5="PASS"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E9">
     <cfRule type="expression" dxfId="0" priority="2">
       <formula>E5="FAIL"</formula>
     </cfRule>

</xml_diff>

<commit_message>
fix: remove local path from Hanoi workbook
</commit_message>
<xml_diff>
--- a/Hanoi/Hanoi-1.0.xlsx
+++ b/Hanoi/Hanoi-1.0.xlsx
@@ -3,12 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Hanoi/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8614F1C1-E031-414D-9764-50EEF05ACB3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF767297-7B80-AF40-BD9B-129997C6A270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15840" xr2:uid="{82D447F9-66A8-4F40-88AB-946121063596}"/>
   </bookViews>
@@ -2062,20 +2057,20 @@
     <xf numFmtId="0" fontId="5" fillId="9" borderId="96" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="97" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="97" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4627,28 +4622,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="34" customHeight="1">
-      <c r="A1" s="134" t="s">
+      <c r="A1" s="132" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="134"/>
-      <c r="C1" s="134"/>
-      <c r="D1" s="134"/>
-      <c r="E1" s="134"/>
-      <c r="F1" s="134"/>
-      <c r="G1" s="134"/>
-      <c r="H1" s="134"/>
+      <c r="B1" s="132"/>
+      <c r="C1" s="132"/>
+      <c r="D1" s="132"/>
+      <c r="E1" s="132"/>
+      <c r="F1" s="132"/>
+      <c r="G1" s="132"/>
+      <c r="H1" s="132"/>
     </row>
     <row r="2" spans="1:8" ht="26" customHeight="1">
-      <c r="A2" s="135" t="s">
+      <c r="A2" s="133" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="135"/>
-      <c r="C2" s="135"/>
-      <c r="D2" s="135"/>
-      <c r="E2" s="135"/>
-      <c r="F2" s="135"/>
-      <c r="G2" s="135"/>
-      <c r="H2" s="135"/>
+      <c r="B2" s="133"/>
+      <c r="C2" s="133"/>
+      <c r="D2" s="133"/>
+      <c r="E2" s="133"/>
+      <c r="F2" s="133"/>
+      <c r="G2" s="133"/>
+      <c r="H2" s="133"/>
     </row>
     <row r="3" spans="1:8" ht="10" customHeight="1">
       <c r="A3" s="121"/>
@@ -4661,52 +4656,52 @@
       <c r="H3" s="121"/>
     </row>
     <row r="4" spans="1:8" ht="24" customHeight="1">
-      <c r="A4" s="133" t="s">
+      <c r="A4" s="134" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="133"/>
-      <c r="C4" s="133"/>
-      <c r="D4" s="133"/>
-      <c r="E4" s="133"/>
-      <c r="F4" s="133"/>
-      <c r="G4" s="133"/>
-      <c r="H4" s="133"/>
+      <c r="B4" s="134"/>
+      <c r="C4" s="134"/>
+      <c r="D4" s="134"/>
+      <c r="E4" s="134"/>
+      <c r="F4" s="134"/>
+      <c r="G4" s="134"/>
+      <c r="H4" s="134"/>
     </row>
     <row r="5" spans="1:8" ht="24" customHeight="1">
-      <c r="A5" s="132" t="s">
+      <c r="A5" s="131" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="132"/>
-      <c r="C5" s="132"/>
-      <c r="D5" s="132"/>
-      <c r="E5" s="132"/>
-      <c r="F5" s="132"/>
-      <c r="G5" s="132"/>
-      <c r="H5" s="132"/>
+      <c r="B5" s="131"/>
+      <c r="C5" s="131"/>
+      <c r="D5" s="131"/>
+      <c r="E5" s="131"/>
+      <c r="F5" s="131"/>
+      <c r="G5" s="131"/>
+      <c r="H5" s="131"/>
     </row>
     <row r="6" spans="1:8" ht="24" customHeight="1">
-      <c r="A6" s="132" t="s">
+      <c r="A6" s="131" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="132"/>
-      <c r="C6" s="132"/>
-      <c r="D6" s="132"/>
-      <c r="E6" s="132"/>
-      <c r="F6" s="132"/>
-      <c r="G6" s="132"/>
-      <c r="H6" s="132"/>
+      <c r="B6" s="131"/>
+      <c r="C6" s="131"/>
+      <c r="D6" s="131"/>
+      <c r="E6" s="131"/>
+      <c r="F6" s="131"/>
+      <c r="G6" s="131"/>
+      <c r="H6" s="131"/>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1">
-      <c r="A7" s="132" t="s">
+      <c r="A7" s="131" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="132"/>
-      <c r="C7" s="132"/>
-      <c r="D7" s="132"/>
-      <c r="E7" s="132"/>
-      <c r="F7" s="132"/>
-      <c r="G7" s="132"/>
-      <c r="H7" s="132"/>
+      <c r="B7" s="131"/>
+      <c r="C7" s="131"/>
+      <c r="D7" s="131"/>
+      <c r="E7" s="131"/>
+      <c r="F7" s="131"/>
+      <c r="G7" s="131"/>
+      <c r="H7" s="131"/>
     </row>
     <row r="8" spans="1:8" ht="10" customHeight="1">
       <c r="A8" s="121"/>
@@ -4719,28 +4714,28 @@
       <c r="H8" s="121"/>
     </row>
     <row r="9" spans="1:8" ht="24" customHeight="1">
-      <c r="A9" s="133" t="s">
+      <c r="A9" s="134" t="s">
         <v>43</v>
       </c>
-      <c r="B9" s="133"/>
-      <c r="C9" s="133"/>
-      <c r="D9" s="133"/>
-      <c r="E9" s="133"/>
-      <c r="F9" s="133"/>
-      <c r="G9" s="133"/>
-      <c r="H9" s="133"/>
+      <c r="B9" s="134"/>
+      <c r="C9" s="134"/>
+      <c r="D9" s="134"/>
+      <c r="E9" s="134"/>
+      <c r="F9" s="134"/>
+      <c r="G9" s="134"/>
+      <c r="H9" s="134"/>
     </row>
     <row r="10" spans="1:8" ht="40" customHeight="1">
-      <c r="A10" s="132" t="s">
+      <c r="A10" s="131" t="s">
         <v>44</v>
       </c>
-      <c r="B10" s="132"/>
-      <c r="C10" s="132"/>
-      <c r="D10" s="132"/>
-      <c r="E10" s="132"/>
-      <c r="F10" s="132"/>
-      <c r="G10" s="132"/>
-      <c r="H10" s="132"/>
+      <c r="B10" s="131"/>
+      <c r="C10" s="131"/>
+      <c r="D10" s="131"/>
+      <c r="E10" s="131"/>
+      <c r="F10" s="131"/>
+      <c r="G10" s="131"/>
+      <c r="H10" s="131"/>
     </row>
     <row r="11" spans="1:8" ht="10" customHeight="1">
       <c r="A11" s="121"/>
@@ -4753,52 +4748,52 @@
       <c r="H11" s="121"/>
     </row>
     <row r="12" spans="1:8" ht="24" customHeight="1">
-      <c r="A12" s="133" t="s">
+      <c r="A12" s="134" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="133"/>
-      <c r="C12" s="133"/>
-      <c r="D12" s="133"/>
-      <c r="E12" s="133"/>
-      <c r="F12" s="133"/>
-      <c r="G12" s="133"/>
-      <c r="H12" s="133"/>
+      <c r="B12" s="134"/>
+      <c r="C12" s="134"/>
+      <c r="D12" s="134"/>
+      <c r="E12" s="134"/>
+      <c r="F12" s="134"/>
+      <c r="G12" s="134"/>
+      <c r="H12" s="134"/>
     </row>
     <row r="13" spans="1:8" ht="26" customHeight="1">
-      <c r="A13" s="132" t="s">
+      <c r="A13" s="131" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="132"/>
-      <c r="C13" s="132"/>
-      <c r="D13" s="132"/>
-      <c r="E13" s="132"/>
-      <c r="F13" s="132"/>
-      <c r="G13" s="132"/>
-      <c r="H13" s="132"/>
+      <c r="B13" s="131"/>
+      <c r="C13" s="131"/>
+      <c r="D13" s="131"/>
+      <c r="E13" s="131"/>
+      <c r="F13" s="131"/>
+      <c r="G13" s="131"/>
+      <c r="H13" s="131"/>
     </row>
     <row r="14" spans="1:8" ht="24" customHeight="1">
-      <c r="A14" s="132" t="s">
+      <c r="A14" s="131" t="s">
         <v>47</v>
       </c>
-      <c r="B14" s="132"/>
-      <c r="C14" s="132"/>
-      <c r="D14" s="132"/>
-      <c r="E14" s="132"/>
-      <c r="F14" s="132"/>
-      <c r="G14" s="132"/>
-      <c r="H14" s="132"/>
+      <c r="B14" s="131"/>
+      <c r="C14" s="131"/>
+      <c r="D14" s="131"/>
+      <c r="E14" s="131"/>
+      <c r="F14" s="131"/>
+      <c r="G14" s="131"/>
+      <c r="H14" s="131"/>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1">
-      <c r="A15" s="132" t="s">
+      <c r="A15" s="131" t="s">
         <v>48</v>
       </c>
-      <c r="B15" s="132"/>
-      <c r="C15" s="132"/>
-      <c r="D15" s="132"/>
-      <c r="E15" s="132"/>
-      <c r="F15" s="132"/>
-      <c r="G15" s="132"/>
-      <c r="H15" s="132"/>
+      <c r="B15" s="131"/>
+      <c r="C15" s="131"/>
+      <c r="D15" s="131"/>
+      <c r="E15" s="131"/>
+      <c r="F15" s="131"/>
+      <c r="G15" s="131"/>
+      <c r="H15" s="131"/>
     </row>
     <row r="16" spans="1:8" ht="10" customHeight="1">
       <c r="A16" s="121"/>
@@ -4811,40 +4806,40 @@
       <c r="H16" s="121"/>
     </row>
     <row r="17" spans="1:8" ht="24" customHeight="1">
-      <c r="A17" s="133" t="s">
+      <c r="A17" s="134" t="s">
         <v>49</v>
       </c>
-      <c r="B17" s="133"/>
-      <c r="C17" s="133"/>
-      <c r="D17" s="133"/>
-      <c r="E17" s="133"/>
-      <c r="F17" s="133"/>
-      <c r="G17" s="133"/>
-      <c r="H17" s="133"/>
+      <c r="B17" s="134"/>
+      <c r="C17" s="134"/>
+      <c r="D17" s="134"/>
+      <c r="E17" s="134"/>
+      <c r="F17" s="134"/>
+      <c r="G17" s="134"/>
+      <c r="H17" s="134"/>
     </row>
     <row r="18" spans="1:8" ht="28" customHeight="1">
-      <c r="A18" s="132" t="s">
+      <c r="A18" s="131" t="s">
         <v>50</v>
       </c>
-      <c r="B18" s="132"/>
-      <c r="C18" s="132"/>
-      <c r="D18" s="132"/>
-      <c r="E18" s="132"/>
-      <c r="F18" s="132"/>
-      <c r="G18" s="132"/>
-      <c r="H18" s="132"/>
+      <c r="B18" s="131"/>
+      <c r="C18" s="131"/>
+      <c r="D18" s="131"/>
+      <c r="E18" s="131"/>
+      <c r="F18" s="131"/>
+      <c r="G18" s="131"/>
+      <c r="H18" s="131"/>
     </row>
     <row r="19" spans="1:8" ht="30" customHeight="1">
-      <c r="A19" s="132" t="s">
+      <c r="A19" s="131" t="s">
         <v>51</v>
       </c>
-      <c r="B19" s="132"/>
-      <c r="C19" s="132"/>
-      <c r="D19" s="132"/>
-      <c r="E19" s="132"/>
-      <c r="F19" s="132"/>
-      <c r="G19" s="132"/>
-      <c r="H19" s="132"/>
+      <c r="B19" s="131"/>
+      <c r="C19" s="131"/>
+      <c r="D19" s="131"/>
+      <c r="E19" s="131"/>
+      <c r="F19" s="131"/>
+      <c r="G19" s="131"/>
+      <c r="H19" s="131"/>
     </row>
     <row r="20" spans="1:8" ht="10" customHeight="1">
       <c r="A20" s="121"/>
@@ -4857,64 +4852,64 @@
       <c r="H20" s="121"/>
     </row>
     <row r="21" spans="1:8" ht="24" customHeight="1">
-      <c r="A21" s="133" t="s">
+      <c r="A21" s="134" t="s">
         <v>52</v>
       </c>
-      <c r="B21" s="133"/>
-      <c r="C21" s="133"/>
-      <c r="D21" s="133"/>
-      <c r="E21" s="133"/>
-      <c r="F21" s="133"/>
-      <c r="G21" s="133"/>
-      <c r="H21" s="133"/>
+      <c r="B21" s="134"/>
+      <c r="C21" s="134"/>
+      <c r="D21" s="134"/>
+      <c r="E21" s="134"/>
+      <c r="F21" s="134"/>
+      <c r="G21" s="134"/>
+      <c r="H21" s="134"/>
     </row>
     <row r="22" spans="1:8" ht="26" customHeight="1">
-      <c r="A22" s="132" t="s">
+      <c r="A22" s="131" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="132"/>
-      <c r="C22" s="132"/>
-      <c r="D22" s="132"/>
-      <c r="E22" s="132"/>
-      <c r="F22" s="132"/>
-      <c r="G22" s="132"/>
-      <c r="H22" s="132"/>
+      <c r="B22" s="131"/>
+      <c r="C22" s="131"/>
+      <c r="D22" s="131"/>
+      <c r="E22" s="131"/>
+      <c r="F22" s="131"/>
+      <c r="G22" s="131"/>
+      <c r="H22" s="131"/>
     </row>
     <row r="23" spans="1:8" ht="28" customHeight="1">
-      <c r="A23" s="132" t="s">
+      <c r="A23" s="131" t="s">
         <v>54</v>
       </c>
-      <c r="B23" s="132"/>
-      <c r="C23" s="132"/>
-      <c r="D23" s="132"/>
-      <c r="E23" s="132"/>
-      <c r="F23" s="132"/>
-      <c r="G23" s="132"/>
-      <c r="H23" s="132"/>
+      <c r="B23" s="131"/>
+      <c r="C23" s="131"/>
+      <c r="D23" s="131"/>
+      <c r="E23" s="131"/>
+      <c r="F23" s="131"/>
+      <c r="G23" s="131"/>
+      <c r="H23" s="131"/>
     </row>
     <row r="24" spans="1:8" ht="26" customHeight="1">
-      <c r="A24" s="132" t="s">
+      <c r="A24" s="131" t="s">
         <v>55</v>
       </c>
-      <c r="B24" s="132"/>
-      <c r="C24" s="132"/>
-      <c r="D24" s="132"/>
-      <c r="E24" s="132"/>
-      <c r="F24" s="132"/>
-      <c r="G24" s="132"/>
-      <c r="H24" s="132"/>
+      <c r="B24" s="131"/>
+      <c r="C24" s="131"/>
+      <c r="D24" s="131"/>
+      <c r="E24" s="131"/>
+      <c r="F24" s="131"/>
+      <c r="G24" s="131"/>
+      <c r="H24" s="131"/>
     </row>
     <row r="25" spans="1:8" ht="36" customHeight="1">
-      <c r="A25" s="132" t="s">
+      <c r="A25" s="131" t="s">
         <v>56</v>
       </c>
-      <c r="B25" s="132"/>
-      <c r="C25" s="132"/>
-      <c r="D25" s="132"/>
-      <c r="E25" s="132"/>
-      <c r="F25" s="132"/>
-      <c r="G25" s="132"/>
-      <c r="H25" s="132"/>
+      <c r="B25" s="131"/>
+      <c r="C25" s="131"/>
+      <c r="D25" s="131"/>
+      <c r="E25" s="131"/>
+      <c r="F25" s="131"/>
+      <c r="G25" s="131"/>
+      <c r="H25" s="131"/>
     </row>
     <row r="26" spans="1:8" ht="10" customHeight="1">
       <c r="A26" s="121"/>
@@ -4927,28 +4922,28 @@
       <c r="H26" s="121"/>
     </row>
     <row r="27" spans="1:8" ht="24" customHeight="1">
-      <c r="A27" s="133" t="s">
+      <c r="A27" s="134" t="s">
         <v>57</v>
       </c>
-      <c r="B27" s="133"/>
-      <c r="C27" s="133"/>
-      <c r="D27" s="133"/>
-      <c r="E27" s="133"/>
-      <c r="F27" s="133"/>
-      <c r="G27" s="133"/>
-      <c r="H27" s="133"/>
+      <c r="B27" s="134"/>
+      <c r="C27" s="134"/>
+      <c r="D27" s="134"/>
+      <c r="E27" s="134"/>
+      <c r="F27" s="134"/>
+      <c r="G27" s="134"/>
+      <c r="H27" s="134"/>
     </row>
     <row r="28" spans="1:8" ht="30" customHeight="1">
-      <c r="A28" s="132" t="s">
+      <c r="A28" s="131" t="s">
         <v>58</v>
       </c>
-      <c r="B28" s="132"/>
-      <c r="C28" s="132"/>
-      <c r="D28" s="132"/>
-      <c r="E28" s="132"/>
-      <c r="F28" s="132"/>
-      <c r="G28" s="132"/>
-      <c r="H28" s="132"/>
+      <c r="B28" s="131"/>
+      <c r="C28" s="131"/>
+      <c r="D28" s="131"/>
+      <c r="E28" s="131"/>
+      <c r="F28" s="131"/>
+      <c r="G28" s="131"/>
+      <c r="H28" s="131"/>
     </row>
     <row r="29" spans="1:8" ht="10" customHeight="1">
       <c r="A29" s="121"/>
@@ -4961,49 +4956,50 @@
       <c r="H29" s="121"/>
     </row>
     <row r="30" spans="1:8" ht="24" customHeight="1">
-      <c r="A30" s="133" t="s">
+      <c r="A30" s="134" t="s">
         <v>59</v>
       </c>
-      <c r="B30" s="133"/>
-      <c r="C30" s="133"/>
-      <c r="D30" s="133"/>
-      <c r="E30" s="133"/>
-      <c r="F30" s="133"/>
-      <c r="G30" s="133"/>
-      <c r="H30" s="133"/>
+      <c r="B30" s="134"/>
+      <c r="C30" s="134"/>
+      <c r="D30" s="134"/>
+      <c r="E30" s="134"/>
+      <c r="F30" s="134"/>
+      <c r="G30" s="134"/>
+      <c r="H30" s="134"/>
     </row>
     <row r="31" spans="1:8" ht="34" customHeight="1">
-      <c r="A31" s="132" t="s">
+      <c r="A31" s="131" t="s">
         <v>60</v>
       </c>
-      <c r="B31" s="132"/>
-      <c r="C31" s="132"/>
-      <c r="D31" s="132"/>
-      <c r="E31" s="132"/>
-      <c r="F31" s="132"/>
-      <c r="G31" s="132"/>
-      <c r="H31" s="132"/>
+      <c r="B31" s="131"/>
+      <c r="C31" s="131"/>
+      <c r="D31" s="131"/>
+      <c r="E31" s="131"/>
+      <c r="F31" s="131"/>
+      <c r="G31" s="131"/>
+      <c r="H31" s="131"/>
     </row>
     <row r="32" spans="1:8" ht="30" customHeight="1">
-      <c r="A32" s="131" t="s">
+      <c r="A32" s="135" t="s">
         <v>61</v>
       </c>
-      <c r="B32" s="131"/>
-      <c r="C32" s="131"/>
-      <c r="D32" s="131"/>
-      <c r="E32" s="131"/>
-      <c r="F32" s="131"/>
-      <c r="G32" s="131"/>
-      <c r="H32" s="131"/>
+      <c r="B32" s="135"/>
+      <c r="C32" s="135"/>
+      <c r="D32" s="135"/>
+      <c r="E32" s="135"/>
+      <c r="F32" s="135"/>
+      <c r="G32" s="135"/>
+      <c r="H32" s="135"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A31:H31"/>
     <mergeCell ref="A23:H23"/>
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="A10:H10"/>
@@ -5016,13 +5012,12 @@
     <mergeCell ref="A19:H19"/>
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="A22:H22"/>
-    <mergeCell ref="A32:H32"/>
-    <mergeCell ref="A24:H24"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="A28:H28"/>
-    <mergeCell ref="A30:H30"/>
-    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A6:H6"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>